<commit_message>
feat(v2.1): Serial Number per unit, shown next to every model name
- Server (Code.gs, needs Apps Script Version 8): Products gets column M "Serial"
  appended at the end (written as text, keeps leading zeros; header auto-created;
  old 12-column sheets keep working). prodSerials_() joins serial by slot code
  for pm_dashboard, lookup and all 5 email templates. Registrations unchanged
- Web: snOf/snHtml/snTxt + .sn (regular weight, 12px v1 / 14px v2, 72% opacity of
  the surrounding text colour) next to the model in Tab 2 cards/table, picker,
  Tab 4, card 03, quick-pay modal, Tab 3, PM tables, receipt modal, upload
  preview and dialogs. Export adds "Serial Number" after "Model" (23 fields).
  "Tải file mẫu" now serves the owner's 8-column template. Serial no longer
  copied into the description
- Harness +10 -> 83/83; scenario 20 -> 126/126 default and ?ui=v1; e2e 165

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Mau_Danh_Muc_San_Pham_Internal_Sales.xlsx
+++ b/data/Mau_Danh_Muc_San_Pham_Internal_Sales.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macbook/Documents/antigravity/AI study/LG other/Internal sales platform/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F56907B4-53E5-EA42-A1B5-151D0DA467E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42D1FBBE-641E-C54E-9201-AAD2D7192938}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="37">
   <si>
     <t>WH (Kho)</t>
   </si>
@@ -110,6 +110,27 @@
   </si>
   <si>
     <t>Xước nhẹ,hộp cũ rách</t>
+  </si>
+  <si>
+    <t>SERIAL NUMBER</t>
+  </si>
+  <si>
+    <t>7328194371830</t>
+  </si>
+  <si>
+    <t>4632784283431</t>
+  </si>
+  <si>
+    <t>3243274816322</t>
+  </si>
+  <si>
+    <t>3342347823412</t>
+  </si>
+  <si>
+    <t>0123123178943</t>
+  </si>
+  <si>
+    <t>0012321398180</t>
   </si>
 </sst>
 </file>
@@ -176,7 +197,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -188,6 +209,7 @@
     <xf numFmtId="3" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -490,17 +512,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="14" customWidth="1"/>
-    <col min="3" max="3" width="22" customWidth="1"/>
-    <col min="4" max="5" width="18" customWidth="1"/>
-    <col min="6" max="6" width="20" customWidth="1"/>
-    <col min="7" max="7" width="50" customWidth="1"/>
+    <col min="3" max="4" width="22" customWidth="1"/>
+    <col min="5" max="6" width="18" customWidth="1"/>
+    <col min="7" max="7" width="20" customWidth="1"/>
+    <col min="8" max="8" width="50" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -511,19 +533,22 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>7</v>
       </c>
@@ -533,20 +558,23 @@
       <c r="C2" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="E2" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="E2" s="4">
+      <c r="F2" s="4">
         <v>24900000</v>
       </c>
-      <c r="F2" s="4">
+      <c r="G2" s="4">
         <v>42990000</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="H2" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>10</v>
       </c>
@@ -556,20 +584,23 @@
       <c r="C3" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="E3" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="E3" s="4">
+      <c r="F3" s="4">
         <v>32500000</v>
       </c>
-      <c r="F3" s="4">
+      <c r="G3" s="4">
         <v>54990000</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="H3" s="3" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>13</v>
       </c>
@@ -579,20 +610,23 @@
       <c r="C4" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="E4" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="E4" s="4">
+      <c r="F4" s="4">
         <v>12900000</v>
       </c>
-      <c r="F4" s="4">
+      <c r="G4" s="4">
         <v>21990000</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="H4" s="3" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>7</v>
       </c>
@@ -602,20 +636,23 @@
       <c r="C5" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="E5" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="E5" s="4">
+      <c r="F5" s="4">
         <v>7800000</v>
       </c>
-      <c r="F5" s="4">
+      <c r="G5" s="4">
         <v>13490000</v>
       </c>
-      <c r="G5" s="3" t="s">
+      <c r="H5" s="3" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>10</v>
       </c>
@@ -625,20 +662,23 @@
       <c r="C6" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="E6" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="E6" s="4">
+      <c r="F6" s="4">
         <v>38900000</v>
       </c>
-      <c r="F6" s="4">
+      <c r="G6" s="4">
         <v>68900000</v>
       </c>
-      <c r="G6" s="3" t="s">
+      <c r="H6" s="3" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>13</v>
       </c>
@@ -648,16 +688,19 @@
       <c r="C7" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D7" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="E7" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="E7" s="4">
+      <c r="F7" s="4">
         <v>7200000</v>
       </c>
-      <c r="F7" s="4">
+      <c r="G7" s="4">
         <v>12500000</v>
       </c>
-      <c r="G7" s="3" t="s">
+      <c r="H7" s="3" t="s">
         <v>29</v>
       </c>
     </row>

</xml_diff>